<commit_message>
adding 3 generic tests
</commit_message>
<xml_diff>
--- a/Generic_qa_report/Housing_data.xlsx
+++ b/Generic_qa_report/Housing_data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\git_demo\Generic_qa_report\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A7A9E9E6-EFC2-4F5B-B80A-7061F3C946BE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BF6222FB-B00C-4A66-9AEF-72A28A3BA8C3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" xr2:uid="{AB3678B5-2446-4328-882A-A72900DC8DCC}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" activeTab="1" xr2:uid="{AB3678B5-2446-4328-882A-A72900DC8DCC}"/>
   </bookViews>
   <sheets>
     <sheet name="introduction" sheetId="4" r:id="rId1"/>
@@ -715,26 +715,14 @@
     <t>Publishing confidence intervals is a work in progress</t>
   </si>
   <si>
-    <r>
-      <t xml:space="preserve">These statistics were adapted from data from the Land Registry licensed under the Open Government Licence v.3.0. Detailed information and download links for the Land Registry Price Paid data used in the production of these statistics at </t>
-    </r>
-    <r>
-      <rPr>
-        <u/>
-        <sz val="12"/>
-        <color rgb="FF0070C0"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>https://www.gov.uk/guidance/about-the-price-paid-data</t>
-    </r>
+    <t>These statistics were adapted from data from the Land Registry licensed under the Open Government Licence v.3.0.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="22" x14ac:knownFonts="1">
+  <fonts count="21" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -886,13 +874,6 @@
     <font>
       <sz val="9"/>
       <color theme="1"/>
-      <name val="Arial"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <u/>
-      <sz val="12"/>
-      <color rgb="FF0070C0"/>
       <name val="Arial"/>
       <family val="2"/>
     </font>

</xml_diff>

<commit_message>
adding more data cleaning tests
</commit_message>
<xml_diff>
--- a/Generic_qa_report/Housing_data.xlsx
+++ b/Generic_qa_report/Housing_data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\git_demo\Generic_qa_report\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BF6222FB-B00C-4A66-9AEF-72A28A3BA8C3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A15AE368-C985-47C9-B513-0E0B8CE25B74}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" activeTab="1" xr2:uid="{AB3678B5-2446-4328-882A-A72900DC8DCC}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" xr2:uid="{AB3678B5-2446-4328-882A-A72900DC8DCC}"/>
   </bookViews>
   <sheets>
     <sheet name="introduction" sheetId="4" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2009" uniqueCount="226">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2011" uniqueCount="227">
   <si>
     <t>Code</t>
   </si>
@@ -715,7 +715,10 @@
     <t>Publishing confidence intervals is a work in progress</t>
   </si>
   <si>
-    <t>These statistics were adapted from data from the Land Registry licensed under the Open Government Licence v.3.0.</t>
+    <t>NaN</t>
+  </si>
+  <si>
+    <t>These statistics were adapted from data from the Land Registry licensed under the Open Government Licence v.3.0</t>
   </si>
 </sst>
 </file>
@@ -1696,7 +1699,7 @@
         <v>212</v>
       </c>
       <c r="B3" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.35">
@@ -1900,11 +1903,11 @@
       <c r="D5" s="12">
         <v>3887</v>
       </c>
-      <c r="E5" s="10">
-        <v>1365</v>
-      </c>
-      <c r="F5" s="10">
-        <v>1565</v>
+      <c r="E5" s="10" t="s">
+        <v>225</v>
+      </c>
+      <c r="F5" s="10" t="s">
+        <v>225</v>
       </c>
       <c r="G5" s="10">
         <v>873</v>
@@ -15928,10 +15931,10 @@
         <v>188750</v>
       </c>
       <c r="E53" s="18" t="s">
-        <v>200</v>
+        <v>225</v>
       </c>
       <c r="F53" s="18" t="s">
-        <v>200</v>
+        <v>225</v>
       </c>
       <c r="G53" s="18">
         <v>223750</v>

</xml_diff>